<commit_message>
Remove numbers from RR52
</commit_message>
<xml_diff>
--- a/Excel/v5/UKRR DataSet v5.2.xlsx
+++ b/Excel/v5/UKRR DataSet v5.2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marta.badji\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A4F67A3-49C2-4F6B-88A0-25787A33B6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9B7B4B3-FDA6-4737-B997-85304C02C1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2170" uniqueCount="1175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2176" uniqueCount="1175">
   <si>
     <t>Introduction to UKRR Dataset v5.2</t>
   </si>
@@ -5064,6 +5064,18 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5081,18 +5093,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -12242,46 +12242,47 @@
     <col min="17" max="17" width="32.83203125" customWidth="1"/>
     <col min="18" max="18" width="30.08203125" customWidth="1"/>
     <col min="21" max="21" width="32.5" customWidth="1"/>
+    <col min="23" max="23" width="15.58203125" customWidth="1"/>
     <col min="24" max="24" width="17.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:24" s="98" customFormat="1" ht="23.5">
-      <c r="A2" s="256" t="s">
+      <c r="A2" s="250" t="s">
         <v>117</v>
       </c>
-      <c r="B2" s="256"/>
-      <c r="C2" s="256"/>
+      <c r="B2" s="250"/>
+      <c r="C2" s="250"/>
       <c r="D2" s="96"/>
       <c r="E2" s="97" t="s">
         <v>119</v>
       </c>
       <c r="F2" s="97"/>
-      <c r="H2" s="254" t="s">
+      <c r="H2" s="248" t="s">
         <v>662</v>
       </c>
-      <c r="I2" s="254"/>
+      <c r="I2" s="248"/>
       <c r="K2" s="95" t="s">
         <v>663</v>
       </c>
       <c r="L2" s="95"/>
       <c r="M2" s="99"/>
-      <c r="N2" s="254" t="s">
+      <c r="N2" s="248" t="s">
         <v>664</v>
       </c>
-      <c r="O2" s="254"/>
-      <c r="Q2" s="254" t="s">
+      <c r="O2" s="248"/>
+      <c r="Q2" s="248" t="s">
         <v>121</v>
       </c>
-      <c r="R2" s="254"/>
+      <c r="R2" s="248"/>
       <c r="S2" s="100"/>
-      <c r="T2" s="254" t="s">
+      <c r="T2" s="248" t="s">
         <v>123</v>
       </c>
-      <c r="U2" s="254"/>
-      <c r="W2" s="253" t="s">
+      <c r="U2" s="248"/>
+      <c r="W2" s="247" t="s">
         <v>1172</v>
       </c>
-      <c r="X2" s="253"/>
+      <c r="X2" s="247"/>
     </row>
     <row r="3" spans="1:24" ht="23.5">
       <c r="A3" s="62" t="s">
@@ -12314,10 +12315,10 @@
       <c r="B4" s="62"/>
       <c r="C4" s="65"/>
       <c r="D4" s="66"/>
-      <c r="E4" s="255" t="s">
+      <c r="E4" s="249" t="s">
         <v>667</v>
       </c>
-      <c r="F4" s="255"/>
+      <c r="F4" s="249"/>
       <c r="H4" s="121" t="s">
         <v>668</v>
       </c>
@@ -12447,8 +12448,8 @@
       <c r="U6" s="74" t="s">
         <v>687</v>
       </c>
-      <c r="W6" s="187">
-        <v>1</v>
+      <c r="W6" s="188" t="s">
+        <v>146</v>
       </c>
       <c r="X6" s="188" t="s">
         <v>146</v>
@@ -12502,8 +12503,8 @@
       <c r="U7" s="74" t="s">
         <v>699</v>
       </c>
-      <c r="W7" s="187">
-        <v>2</v>
+      <c r="W7" s="188" t="s">
+        <v>557</v>
       </c>
       <c r="X7" s="188" t="s">
         <v>557</v>
@@ -12557,8 +12558,8 @@
       <c r="U8" s="74" t="s">
         <v>710</v>
       </c>
-      <c r="W8" s="187">
-        <v>3</v>
+      <c r="W8" s="188" t="s">
+        <v>1165</v>
       </c>
       <c r="X8" s="188" t="s">
         <v>1165</v>
@@ -12608,8 +12609,8 @@
       <c r="U9" s="74" t="s">
         <v>719</v>
       </c>
-      <c r="W9" s="187">
-        <v>4</v>
+      <c r="W9" s="188" t="s">
+        <v>1166</v>
       </c>
       <c r="X9" s="188" t="s">
         <v>1166</v>
@@ -12659,8 +12660,8 @@
       <c r="U10" s="74" t="s">
         <v>729</v>
       </c>
-      <c r="W10" s="187">
-        <v>5</v>
+      <c r="W10" s="188" t="s">
+        <v>1167</v>
       </c>
       <c r="X10" s="188" t="s">
         <v>1167</v>
@@ -12710,8 +12711,8 @@
       <c r="U11" s="74" t="s">
         <v>739</v>
       </c>
-      <c r="W11" s="187">
-        <v>6</v>
+      <c r="W11" s="188" t="s">
+        <v>1168</v>
       </c>
       <c r="X11" s="188" t="s">
         <v>1168</v>
@@ -15550,7 +15551,7 @@
       <c r="I4" s="210" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="247" t="s">
+      <c r="J4" s="251" t="s">
         <v>19</v>
       </c>
     </row>
@@ -15578,7 +15579,7 @@
       <c r="I5" s="210" t="s">
         <v>18</v>
       </c>
-      <c r="J5" s="248"/>
+      <c r="J5" s="252"/>
     </row>
     <row r="6" spans="1:10" ht="155">
       <c r="A6" s="205" t="s">
@@ -15604,7 +15605,7 @@
       <c r="I6" s="210" t="s">
         <v>18</v>
       </c>
-      <c r="J6" s="248"/>
+      <c r="J6" s="252"/>
     </row>
     <row r="7" spans="1:10" ht="31" customHeight="1">
       <c r="A7" s="205" t="s">
@@ -15630,7 +15631,7 @@
       <c r="I7" s="210" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="248"/>
+      <c r="J7" s="252"/>
     </row>
     <row r="8" spans="1:10" ht="93">
       <c r="A8" s="205" t="s">
@@ -15654,7 +15655,7 @@
       <c r="I8" s="210" t="s">
         <v>18</v>
       </c>
-      <c r="J8" s="248"/>
+      <c r="J8" s="252"/>
     </row>
     <row r="9" spans="1:10" ht="31" customHeight="1">
       <c r="A9" s="205" t="s">
@@ -15676,7 +15677,7 @@
       <c r="I9" s="210" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="248"/>
+      <c r="J9" s="252"/>
     </row>
     <row r="10" spans="1:10" ht="31" customHeight="1">
       <c r="A10" s="205" t="s">
@@ -15700,7 +15701,7 @@
       <c r="I10" s="210" t="s">
         <v>42</v>
       </c>
-      <c r="J10" s="248"/>
+      <c r="J10" s="252"/>
     </row>
     <row r="11" spans="1:10" ht="31">
       <c r="A11" s="205" t="s">
@@ -15724,7 +15725,7 @@
       <c r="I11" s="210" t="s">
         <v>42</v>
       </c>
-      <c r="J11" s="248"/>
+      <c r="J11" s="252"/>
     </row>
     <row r="12" spans="1:10" ht="46.5">
       <c r="A12" s="205" t="s">
@@ -15750,7 +15751,7 @@
       <c r="I12" s="210" t="s">
         <v>42</v>
       </c>
-      <c r="J12" s="248"/>
+      <c r="J12" s="252"/>
     </row>
     <row r="13" spans="1:10" ht="31" customHeight="1">
       <c r="A13" s="205" t="s">
@@ -15774,7 +15775,7 @@
       <c r="I13" s="210" t="s">
         <v>42</v>
       </c>
-      <c r="J13" s="248"/>
+      <c r="J13" s="252"/>
     </row>
     <row r="14" spans="1:10" ht="31" customHeight="1">
       <c r="A14" s="205" t="s">
@@ -15796,7 +15797,7 @@
       <c r="I14" s="210" t="s">
         <v>42</v>
       </c>
-      <c r="J14" s="249"/>
+      <c r="J14" s="253"/>
     </row>
     <row r="15" spans="1:10" ht="31">
       <c r="A15" s="185" t="s">
@@ -15822,7 +15823,7 @@
       <c r="I15" s="193" t="s">
         <v>18</v>
       </c>
-      <c r="J15" s="250" t="s">
+      <c r="J15" s="254" t="s">
         <v>57</v>
       </c>
     </row>
@@ -15850,7 +15851,7 @@
       <c r="I16" s="193" t="s">
         <v>18</v>
       </c>
-      <c r="J16" s="251"/>
+      <c r="J16" s="255"/>
     </row>
     <row r="17" spans="1:10" ht="155">
       <c r="A17" s="185" t="s">
@@ -15876,7 +15877,7 @@
       <c r="I17" s="193" t="s">
         <v>18</v>
       </c>
-      <c r="J17" s="251"/>
+      <c r="J17" s="255"/>
     </row>
     <row r="18" spans="1:10" ht="31" customHeight="1">
       <c r="A18" s="185" t="s">
@@ -15900,7 +15901,7 @@
       <c r="I18" s="193" t="s">
         <v>18</v>
       </c>
-      <c r="J18" s="251"/>
+      <c r="J18" s="255"/>
     </row>
     <row r="19" spans="1:10" ht="77.5">
       <c r="A19" s="185" t="s">
@@ -15924,7 +15925,7 @@
       <c r="I19" s="193" t="s">
         <v>18</v>
       </c>
-      <c r="J19" s="251"/>
+      <c r="J19" s="255"/>
     </row>
     <row r="20" spans="1:10" ht="31" customHeight="1">
       <c r="A20" s="185" t="s">
@@ -15946,7 +15947,7 @@
       <c r="I20" s="193" t="s">
         <v>18</v>
       </c>
-      <c r="J20" s="251"/>
+      <c r="J20" s="255"/>
     </row>
     <row r="21" spans="1:10" ht="118" customHeight="1">
       <c r="A21" s="241" t="s">
@@ -15996,7 +15997,7 @@
       <c r="I22" s="193" t="s">
         <v>42</v>
       </c>
-      <c r="J22" s="251" t="s">
+      <c r="J22" s="255" t="s">
         <v>69</v>
       </c>
     </row>
@@ -16024,7 +16025,7 @@
       <c r="I23" s="193" t="s">
         <v>42</v>
       </c>
-      <c r="J23" s="251"/>
+      <c r="J23" s="255"/>
     </row>
     <row r="24" spans="1:10" ht="31" customHeight="1">
       <c r="A24" s="185" t="s">
@@ -16048,7 +16049,7 @@
       <c r="I24" s="193" t="s">
         <v>42</v>
       </c>
-      <c r="J24" s="251"/>
+      <c r="J24" s="255"/>
     </row>
     <row r="25" spans="1:10" ht="31" customHeight="1">
       <c r="A25" s="185" t="s">
@@ -16070,7 +16071,7 @@
       <c r="I25" s="193" t="s">
         <v>42</v>
       </c>
-      <c r="J25" s="252"/>
+      <c r="J25" s="256"/>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="185" t="s">

</xml_diff>